<commit_message>
Branch Ops: kotak pilihan di Ubah TBO, ejaan baku jenis_rekening, Dikecualikan jadi Tidak ada TBO, perkakas disk VPS
</commit_message>
<xml_diff>
--- a/contoh/Template-03-Data-TBO.xlsx
+++ b/contoh/Template-03-Data-TBO.xlsx
@@ -628,7 +628,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Perusahaan (Non Perorangan)</t>
+          <t>Non Perorangan (Perusahaan)</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Pemindahbukuan</t>
+          <t>Pemindah-bukuan</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Perusahaan (Non Perorangan)</t>
+          <t>Non Perorangan (Perusahaan)</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -964,11 +964,11 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="L4:L500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Jenis Rekening tidak dikenal" error="Nilai tidak dikenal. Pilih salah satu dari daftar - ejaan yang berbeda akan membuat baris ini tidak terhitung di dashboard." promptTitle="Jenis Rekening" prompt="Pilih dari daftar: Perorangan / Perusahaan (Non Perorangan)" type="list">
-      <formula1>"Perorangan,Perusahaan (Non Perorangan)"</formula1>
+    <dataValidation sqref="L4:L500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Jenis Rekening tidak dikenal" error="Nilai tidak dikenal. Pilih salah satu dari daftar - ejaan yang berbeda akan membuat baris ini tidak terhitung di dashboard." promptTitle="Jenis Rekening" prompt="Pilih dari daftar: Perorangan / Non Perorangan (Perusahaan)" type="list">
+      <formula1>"Perorangan,Non Perorangan (Perusahaan)"</formula1>
     </dataValidation>
-    <dataValidation sqref="M4:M500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Jenis Setoran tidak dikenal" error="Nilai tidak dikenal. Pilih salah satu dari daftar - ejaan yang berbeda akan membuat baris ini tidak terhitung di dashboard." promptTitle="Jenis Setoran" prompt="Pilih dari daftar: Transfer / Tunai / Pemindahbukuan" type="list">
-      <formula1>"Transfer,Tunai,Pemindahbukuan"</formula1>
+    <dataValidation sqref="M4:M500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Jenis Setoran tidak dikenal" error="Nilai tidak dikenal. Pilih salah satu dari daftar - ejaan yang berbeda akan membuat baris ini tidak terhitung di dashboard." promptTitle="Jenis Setoran" prompt="Pilih dari daftar: Tunai / Transfer / Pemindah-bukuan" type="list">
+      <formula1>"Tunai,Transfer,Pemindah-bukuan"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>